<commit_message>
Corrida | GLO-BARC | 2026-03-19 12:06:23.256395
</commit_message>
<xml_diff>
--- a/indicadores/GLO-BARC_out.xlsx
+++ b/indicadores/GLO-BARC_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">11/03/2026</t>
+    <t xml:space="preserve">19/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | GLO-BARC | 2026-06-17 11:28:33.632941
</commit_message>
<xml_diff>
--- a/indicadores/GLO-BARC_out.xlsx
+++ b/indicadores/GLO-BARC_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="561">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mundo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">11/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2193,9 +2199,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2206,7 +2216,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2220,7 +2230,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2236,7 +2246,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2264,7 +2274,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2278,7 +2288,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2306,7 +2316,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2320,7 +2330,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2334,7 +2344,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2348,7 +2358,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2364,7 +2374,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2378,7 +2388,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2526,10 +2536,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2542,10 +2552,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2569,66 +2579,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>104.445794597301</v>
@@ -2681,7 +2691,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>101.448092126859</v>
@@ -2738,7 +2748,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>101.378229221773</v>
@@ -2795,7 +2805,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>99.3427574908946</v>
@@ -2852,7 +2862,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>97.0972499181916</v>
@@ -2909,7 +2919,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>96.6532232867326</v>
@@ -2966,7 +2976,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>96.6866522136701</v>
@@ -3023,7 +3033,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>96.3401933467361</v>
@@ -3080,7 +3090,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>96.9598833532042</v>
@@ -3137,7 +3147,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>96.5926074593325</v>
@@ -3194,7 +3204,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>96.998389230338</v>
@@ -3251,7 +3261,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>98.2484352096161</v>
@@ -3308,7 +3318,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>98.7319589544961</v>
@@ -3367,7 +3377,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>99.2832545348978</v>
@@ -3426,7 +3436,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>96.0110824587256</v>
@@ -3485,7 +3495,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>94.7559395708324</v>
@@ -3544,7 +3554,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>97.2292410815276</v>
@@ -3603,7 +3613,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>97.9701683031738</v>
@@ -3662,7 +3672,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>98.6231264949242</v>
@@ -3721,7 +3731,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>97.0686681272037</v>
@@ -3780,7 +3790,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>93.9469470895703</v>
@@ -3839,7 +3849,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>97.9142827563112</v>
@@ -3898,7 +3908,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>98.9846598949872</v>
@@ -3957,7 +3967,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>102.356500618961</v>
@@ -4016,7 +4026,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>106.317164557787</v>
@@ -4075,7 +4085,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>105.106887632704</v>
@@ -4134,7 +4144,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>107.491697797525</v>
@@ -4193,7 +4203,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>107.304043314839</v>
@@ -4252,7 +4262,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>102.685117215129</v>
@@ -4311,7 +4321,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>103.950538081717</v>
@@ -4370,7 +4380,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>102.75707306629</v>
@@ -4429,7 +4439,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>104.623255473208</v>
@@ -4488,7 +4498,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>106.849448589713</v>
@@ -4547,7 +4557,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>109.210605059035</v>
@@ -4606,7 +4616,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>108.234237614798</v>
@@ -4665,7 +4675,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>109.472283909605</v>
@@ -4724,7 +4734,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>107.604652880311</v>
@@ -4783,7 +4793,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>107.127758790271</v>
@@ -4842,7 +4852,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>106.343297739352</v>
@@ -4901,7 +4911,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>109.718413665369</v>
@@ -4960,7 +4970,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>106.952873103445</v>
@@ -5019,7 +5029,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>104.870195384701</v>
@@ -5078,7 +5088,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>102.381510451989</v>
@@ -5137,7 +5147,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>97.0911295453409</v>
@@ -5196,7 +5206,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>95.3345769465366</v>
@@ -5255,7 +5265,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>100.437495101568</v>
@@ -5314,7 +5324,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>90.2467820593769</v>
@@ -5373,7 +5383,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>88.2225302796144</v>
@@ -5432,7 +5442,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>88.8259923422892</v>
@@ -5491,7 +5501,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>84.6633473373831</v>
@@ -5550,7 +5560,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>89.9807987239214</v>
@@ -5609,7 +5619,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>88.9140151050072</v>
@@ -5668,7 +5678,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>88.4908745414479</v>
@@ -5727,7 +5737,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>87.0189643121144</v>
@@ -5786,7 +5796,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>88.8350080554504</v>
@@ -5845,7 +5855,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>91.7338121732786</v>
@@ -5904,7 +5914,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>90.4591707321464</v>
@@ -5963,7 +5973,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>86.8519521769362</v>
@@ -6022,7 +6032,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>88.5965779989032</v>
@@ -6081,7 +6091,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>87.6444598973637</v>
@@ -6140,7 +6150,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>85.7401237631956</v>
@@ -6199,7 +6209,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>89.0245818486251</v>
@@ -6258,7 +6268,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>87.3733679278852</v>
@@ -6317,7 +6327,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>85.0054629943614</v>
@@ -6376,7 +6386,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>91.8238319377074</v>
@@ -6435,7 +6445,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>91.8075836496693</v>
@@ -6494,7 +6504,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>93.2395346641583</v>
@@ -6553,7 +6563,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>93.8184317957976</v>
@@ -6612,7 +6622,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>95.7803328286636</v>
@@ -6671,7 +6681,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>99.2583773981713</v>
@@ -6730,7 +6740,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>97.295167694288</v>
@@ -6789,7 +6799,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>94.4251286287993</v>
@@ -6848,7 +6858,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>87.5434826028659</v>
@@ -6907,7 +6917,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>84.8809876991308</v>
@@ -6966,7 +6976,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>82.9671433924195</v>
@@ -7025,7 +7035,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>82.4930958877384</v>
@@ -7084,7 +7094,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>98.6372324138238</v>
@@ -7143,7 +7153,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>99.2323629809849</v>
@@ -7202,7 +7212,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>94.8373560853877</v>
@@ -7261,7 +7271,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>95.1855345738226</v>
@@ -7320,7 +7330,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>97.767109051091</v>
@@ -7379,7 +7389,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>95.0465287963129</v>
@@ -7438,7 +7448,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>98.6512214737166</v>
@@ -7497,7 +7507,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>98.7863454087043</v>
@@ -7556,7 +7566,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>107.994147007436</v>
@@ -7615,7 +7625,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>105.035062286003</v>
@@ -7674,7 +7684,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>106.91265076196</v>
@@ -7733,7 +7743,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>98.0078644112507</v>
@@ -7792,7 +7802,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>110.608003832719</v>
@@ -7851,7 +7861,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>121.677923364256</v>
@@ -7910,7 +7920,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>127.085237810247</v>
@@ -7969,7 +7979,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>127.401504829898</v>
@@ -8028,7 +8038,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>127.048961040972</v>
@@ -8087,7 +8097,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>132.628781084161</v>
@@ -8146,7 +8156,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>128.941213662001</v>
@@ -8205,7 +8215,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>126.640812676626</v>
@@ -8264,7 +8274,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>128.857433495813</v>
@@ -8323,7 +8333,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>130.415396824834</v>
@@ -8382,7 +8392,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>123.548200934501</v>
@@ -8441,7 +8451,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>133.672974791069</v>
@@ -8500,7 +8510,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>131.301401639332</v>
@@ -8559,7 +8569,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>119.851343895032</v>
@@ -8618,7 +8628,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>120.313353282457</v>
@@ -8677,7 +8687,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>121.836670600796</v>
@@ -8736,7 +8746,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>113.125477618456</v>
@@ -8795,7 +8805,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>111.529091352494</v>
@@ -8854,7 +8864,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>109.754806166907</v>
@@ -8913,7 +8923,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>104.600618464785</v>
@@ -8972,7 +8982,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>99.8942012853812</v>
@@ -9031,7 +9041,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>92.2788958257087</v>
@@ -9090,7 +9100,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>88.2402948387227</v>
@@ -9149,7 +9159,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>84.1404584746729</v>
@@ -9208,7 +9218,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>82.6444281975089</v>
@@ -9267,7 +9277,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>81.0348813194045</v>
@@ -9326,7 +9336,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>81.8941704871275</v>
@@ -9385,7 +9395,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>79.1650216998059</v>
@@ -9444,7 +9454,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>84.0516572408255</v>
@@ -9503,7 +9513,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>77.292363421456</v>
@@ -9562,7 +9572,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>79.4030195820186</v>
@@ -9621,7 +9631,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>80.6452565518936</v>
@@ -9680,7 +9690,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>86.3349852284511</v>
@@ -9739,7 +9749,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>89.2478085883925</v>
@@ -9798,7 +9808,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>96.4365197551881</v>
@@ -9857,7 +9867,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>105.180543327914</v>
@@ -9916,7 +9926,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>108.000590287278</v>
@@ -9975,7 +9985,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>108.224374839515</v>
@@ -10034,7 +10044,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>106.486001897879</v>
@@ -10093,7 +10103,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>105.476760832546</v>
@@ -10152,7 +10162,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>102.672145276865</v>
@@ -10211,7 +10221,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>104.398086627081</v>
@@ -10270,7 +10280,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>102.431106264618</v>
@@ -10329,7 +10339,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>103.150302023078</v>
@@ -10388,7 +10398,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>100.321501878734</v>
@@ -10447,7 +10457,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>99.6725780274798</v>
@@ -10506,7 +10516,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>97.370291172519</v>
@@ -10565,7 +10575,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>93.7097904740426</v>
@@ -10624,7 +10634,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>91.5794187629895</v>
@@ -10683,7 +10693,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>91.2726838190327</v>
@@ -10742,7 +10752,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>94.1774078990242</v>
@@ -10801,7 +10811,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>97.5704681421492</v>
@@ -10860,7 +10870,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>102.080446623804</v>
@@ -10919,7 +10929,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>104.698863976246</v>
@@ -10978,7 +10988,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>112.436862214412</v>
@@ -11037,7 +11047,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>110.672902990466</v>
@@ -11096,7 +11106,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>114.739973387293</v>
@@ -11155,7 +11165,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>112.672182141961</v>
@@ -11214,7 +11224,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>113.349498965657</v>
@@ -11273,7 +11283,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>113.947674740715</v>
@@ -11332,7 +11342,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>119.479832592983</v>
@@ -11391,7 +11401,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>116.787388486323</v>
@@ -11450,7 +11460,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>117.580193498621</v>
@@ -11509,7 +11519,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>115.026546886994</v>
@@ -11568,7 +11578,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>114.161517089434</v>
@@ -11627,7 +11637,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>112.242133728354</v>
@@ -11686,7 +11696,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>106.864486164825</v>
@@ -11745,7 +11755,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>103.84221779248</v>
@@ -11804,7 +11814,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>103.781117474712</v>
@@ -11863,7 +11873,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>108.494171134745</v>
@@ -11922,7 +11932,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>108.2242822304</v>
@@ -11981,7 +11991,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>107.40898365468</v>
@@ -12040,7 +12050,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>101.900324523753</v>
@@ -12099,7 +12109,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>101.522201821372</v>
@@ -12158,7 +12168,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>102.555146142342</v>
@@ -12217,7 +12227,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>103.221680402492</v>
@@ -12276,7 +12286,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>104.975348240847</v>
@@ -12335,7 +12345,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>106.250412987508</v>
@@ -12394,7 +12404,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>107.425969685768</v>
@@ -12453,7 +12463,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>109.262147136146</v>
@@ -12512,7 +12522,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>110.50093283267</v>
@@ -12571,7 +12581,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>111.221209133669</v>
@@ -12630,7 +12640,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>110.190914926105</v>
@@ -12689,7 +12699,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>109.703031259192</v>
@@ -12748,7 +12758,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>112.336988671547</v>
@@ -12807,7 +12817,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>111.523035475205</v>
@@ -12866,7 +12876,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>109.667970977504</v>
@@ -12925,7 +12935,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>107.213773908909</v>
@@ -12984,7 +12994,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>108.20525256857</v>
@@ -13043,7 +13053,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>108.671035640542</v>
@@ -13102,7 +13112,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>111.726735450257</v>
@@ -13161,7 +13171,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>112.900213299967</v>
@@ -13220,7 +13230,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>112.600149061965</v>
@@ -13279,7 +13289,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>112.296691664415</v>
@@ -13338,7 +13348,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>112.205966372001</v>
@@ -13397,7 +13407,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>110.988203926285</v>
@@ -13456,7 +13466,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>108.642384999338</v>
@@ -13515,7 +13525,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>107.761484611516</v>
@@ -13574,7 +13584,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>110.014338542303</v>
@@ -13633,7 +13643,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>109.758544992687</v>
@@ -13692,7 +13702,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>107.853936898166</v>
@@ -13751,7 +13761,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>109.908807698697</v>
@@ -13810,7 +13820,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>107.569331985916</v>
@@ -13869,7 +13879,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>107.402835499431</v>
@@ -13928,7 +13938,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>105.476854553537</v>
@@ -13987,7 +13997,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>103.430712018168</v>
@@ -14046,7 +14056,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>100.609549650002</v>
@@ -14105,7 +14115,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>100.592534964206</v>
@@ -14164,7 +14174,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>97.8243859757902</v>
@@ -14223,7 +14233,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>92.6078392601395</v>
@@ -14282,7 +14292,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>92.5340416909968</v>
@@ -14341,7 +14351,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>88.4648545812303</v>
@@ -14400,7 +14410,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>86.0113974782681</v>
@@ -14459,7 +14469,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>83.8052082540607</v>
@@ -14518,7 +14528,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>68.230425612145</v>
@@ -14577,7 +14587,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>54.6617884813989</v>
@@ -14636,7 +14646,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>53.2058590927963</v>
@@ -14695,7 +14705,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>52.666931763131</v>
@@ -14754,7 +14764,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>53.6275607758631</v>
@@ -14813,7 +14823,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>60.1453554508246</v>
@@ -14872,7 +14882,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>67.3679609863537</v>
@@ -14931,7 +14941,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>75.8121203383833</v>
@@ -14990,7 +15000,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>81.3281919610933</v>
@@ -15049,7 +15059,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>87.7294306481488</v>
@@ -15108,7 +15118,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>96.4790248624811</v>
@@ -15167,7 +15177,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>95.6725553467697</v>
@@ -15226,7 +15236,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>104.258071008312</v>
@@ -15285,7 +15295,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>110.95935199278</v>
@@ -15344,7 +15354,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>113.289770981946</v>
@@ -15403,7 +15413,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>114.925256378527</v>
@@ -15462,7 +15472,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>116.34941514248</v>
@@ -15521,7 +15531,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>117.505155811096</v>
@@ -15580,7 +15590,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>117.527089655011</v>
@@ -15639,7 +15649,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>118.153081103497</v>
@@ -15698,7 +15708,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>114.132091939292</v>
@@ -15757,7 +15767,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>111.982004444883</v>
@@ -15816,7 +15826,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>108.453584871844</v>
@@ -15875,7 +15885,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>109.9381940909</v>
@@ -15934,7 +15944,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>109.586845203528</v>
@@ -15993,7 +16003,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>112.750654507599</v>
@@ -16052,7 +16062,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>113.192037446997</v>
@@ -16111,7 +16121,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>110.77885427831</v>
@@ -16170,7 +16180,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>113.277765444471</v>
@@ -16229,7 +16239,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>108.049240466367</v>
@@ -16288,7 +16298,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>104.163751585839</v>
@@ -16347,7 +16357,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>100.472058877118</v>
@@ -16406,7 +16416,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>99.2689607855336</v>
@@ -16465,7 +16475,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>98.7337103576046</v>
@@ -16524,7 +16534,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>96.4606896739629</v>
@@ -16583,7 +16593,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>95.1578679531183</v>
@@ -16642,7 +16652,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>94.7644420395642</v>
@@ -16701,7 +16711,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>92.7373773741805</v>
@@ -16760,7 +16770,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>93.8982869270673</v>
@@ -16819,7 +16829,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>93.6416215181062</v>
@@ -16878,7 +16888,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>96.514653702237</v>
@@ -16937,7 +16947,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>98.174450027307</v>
@@ -16996,7 +17006,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>97.0388528263008</v>
@@ -17055,7 +17065,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>94.3889895647551</v>
@@ -17114,7 +17124,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>93.6463932158415</v>
@@ -17173,7 +17183,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>89.6457357276217</v>
@@ -17232,7 +17242,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>91.0101864851882</v>
@@ -17291,7 +17301,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>89.6758757688225</v>
@@ -17350,7 +17360,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>86.5885002881582</v>
@@ -17409,7 +17419,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>86.3514079529228</v>
@@ -17468,7 +17478,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>89.1575561085984</v>
@@ -17527,7 +17537,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>90.7880353800031</v>
@@ -17586,7 +17596,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>92.5010109186665</v>
@@ -17645,7 +17655,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>94.0130045827219</v>
@@ -17704,7 +17714,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>91.8826787084403</v>
@@ -17763,7 +17773,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>95.7888048296788</v>
@@ -17822,7 +17832,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>97.7753203169492</v>
@@ -17881,7 +17891,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>98.9337180371906</v>
@@ -17940,7 +17950,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>102.142348478128</v>
@@ -17999,7 +18009,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>104.486763608179</v>
@@ -18058,7 +18068,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>105.79349243856</v>
@@ -18117,7 +18127,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>106.389411363678</v>
@@ -18176,7 +18186,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>104.692812794917</v>
@@ -18235,7 +18245,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>107.28002483536</v>
@@ -18294,7 +18304,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>104.899125907243</v>
@@ -18353,7 +18363,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>103.054353543986</v>
@@ -18412,7 +18422,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>105.25203208406</v>
@@ -18471,7 +18481,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>103.983509601017</v>
@@ -18530,7 +18540,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>103.197210179564</v>
@@ -18589,7 +18599,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>104.781477072666</v>
@@ -18648,7 +18658,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>103.810170440028</v>
@@ -18707,7 +18717,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>103.328621394217</v>
@@ -18766,7 +18776,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>103.784638050218</v>
@@ -18825,7 +18835,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>102.834163160746</v>
@@ -18884,7 +18894,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>99.6985774275286</v>
@@ -18943,7 +18953,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>98.3896279896789</v>
@@ -19002,7 +19012,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>99.0040563131338</v>
@@ -19061,7 +19071,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>98.3234360829448</v>
@@ -19120,7 +19130,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>99.9830767983371</v>
@@ -19179,7 +19189,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>99.4190744063282</v>
@@ -19238,7 +19248,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>99.0678124188773</v>
@@ -19297,7 +19307,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>99.6169370745949</v>
@@ -19356,7 +19366,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>97.4413860178873</v>
@@ -19415,7 +19425,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>96.2989647046471</v>
@@ -19474,7 +19484,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>97.5040949558958</v>
@@ -19533,7 +19543,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>97.0834635397958</v>
@@ -19592,7 +19602,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>97.366356801315</v>
@@ -19651,7 +19661,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>94.6603659768132</v>
@@ -19710,7 +19720,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>92.7184419554394</v>
@@ -19769,7 +19779,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>94.8781387541992</v>
@@ -19828,7 +19838,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>95.9406043223245</v>
@@ -19887,7 +19897,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>95.1544877972297</v>
@@ -19946,7 +19956,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>96.8299232879254</v>
@@ -20005,7 +20015,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>97.4543628031828</v>
@@ -20064,7 +20074,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>99.1473064743428</v>
@@ -20123,7 +20133,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>99.5757600675505</v>
@@ -20182,7 +20192,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>101.027525726996</v>
@@ -20241,7 +20251,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>102.857449010591</v>
@@ -20300,7 +20310,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>105.354748382157</v>
@@ -20359,7 +20369,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>108.671286330834</v>
@@ -20418,7 +20428,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>110.588914609216</v>
@@ -20477,7 +20487,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>111.103247409411</v>
@@ -20536,7 +20546,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>110.983842630967</v>
@@ -20595,7 +20605,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>112.455480040831</v>
@@ -20654,7 +20664,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>113.201539099007</v>
@@ -20713,7 +20723,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>113.497481728202</v>
@@ -20772,7 +20782,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>113.624502717031</v>
@@ -20831,7 +20841,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>116.283562901021</v>
@@ -20890,7 +20900,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>115.897474300329</v>
@@ -20949,7 +20959,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>116.9827975967</v>
@@ -21008,7 +21018,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>117.03021492994</v>
@@ -21067,7 +21077,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>116.789825956046</v>
@@ -21126,7 +21136,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>116.197194983392</v>
@@ -21185,7 +21195,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>114.43228228701</v>
@@ -21244,7 +21254,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>113.428533210706</v>
@@ -21303,7 +21313,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>113.484150106638</v>
@@ -21362,7 +21372,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>111.154261760946</v>
@@ -21421,7 +21431,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>108.44906864656</v>
@@ -21480,7 +21490,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>107.697524866856</v>
@@ -21539,7 +21549,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>106.131849112251</v>
@@ -21598,7 +21608,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>102.699744561792</v>
@@ -21657,7 +21667,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>100.145432471186</v>
@@ -21716,7 +21726,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>98.1700931469112</v>
@@ -21775,7 +21785,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>94.4411860542729</v>
@@ -21834,7 +21844,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>95.2532981681861</v>
@@ -21893,7 +21903,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>98.0812564561919</v>
@@ -21952,7 +21962,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>96.7805968312376</v>
@@ -22011,7 +22021,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>95.9702918523389</v>
@@ -22070,7 +22080,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>95.1878871526249</v>
@@ -22129,7 +22139,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>93.624231746809</v>
@@ -22188,7 +22198,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>92.1288244947055</v>
@@ -22247,7 +22257,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>91.6304144891929</v>
@@ -22306,7 +22316,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>91.1312086913399</v>
@@ -22365,7 +22375,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>93.1321444148159</v>
@@ -22424,7 +22434,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>94.6732168645648</v>
@@ -22483,7 +22493,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>96.5796752729216</v>
@@ -22542,7 +22552,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>81.958477070343</v>
@@ -22601,7 +22611,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>81.0543745686012</v>
@@ -22660,7 +22670,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>55.5232606456555</v>
@@ -22719,7 +22729,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>60.7346700530732</v>
@@ -22778,7 +22788,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>72.1595344437668</v>
@@ -22837,7 +22847,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>85.6605949822612</v>
@@ -22896,7 +22906,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>92.1059092877339</v>
@@ -22955,7 +22965,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>96.0236375367773</v>
@@ -23014,7 +23024,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>103.041137900769</v>
@@ -23073,7 +23083,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>103.054141332927</v>
@@ -23132,7 +23142,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>102.940805077983</v>
@@ -23191,7 +23201,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>104.263802851346</v>
@@ -23250,7 +23260,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>108.137874011968</v>
@@ -23309,7 +23319,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>112.724729986704</v>
@@ -23368,7 +23378,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>126.426687526792</v>
@@ -23427,7 +23437,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>128.000684303357</v>
@@ -23486,7 +23496,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>125.710615209439</v>
@@ -23545,7 +23555,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>121.864178622792</v>
@@ -23604,7 +23614,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>115.972811807703</v>
@@ -23663,7 +23673,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>112.230834870673</v>
@@ -23722,7 +23732,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>110.262622424565</v>
@@ -23781,7 +23791,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>112.376322603819</v>
@@ -23840,7 +23850,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>111.970216791709</v>
@@ -23899,7 +23909,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>109.655496389913</v>
@@ -23958,7 +23968,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>107.588788710651</v>
@@ -24017,7 +24027,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>102.544357266633</v>
@@ -24076,7 +24086,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>99.3614007751258</v>
@@ -24135,7 +24145,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>99.0650036855504</v>
@@ -24194,7 +24204,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>96.5406875023197</v>
@@ -24253,7 +24263,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>92.6560760897401</v>
@@ -24312,7 +24322,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>93.8149524562916</v>
@@ -24371,7 +24381,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>92.4545198494559</v>
@@ -24430,7 +24440,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>90.7302367171814</v>
@@ -24489,7 +24499,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>87.2829919994959</v>
@@ -24548,7 +24558,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>86.9847433824729</v>
@@ -24607,7 +24617,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>89.5994356102579</v>
@@ -24666,7 +24676,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>93.8974871472196</v>
@@ -24725,7 +24735,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>93.9842294163466</v>
@@ -24784,7 +24794,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>95.0611403736899</v>
@@ -24843,7 +24853,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>93.6550804151918</v>
@@ -24902,7 +24912,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>94.0847658490591</v>
@@ -24961,7 +24971,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>95.4561148223926</v>
@@ -25020,7 +25030,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>94.1032506581174</v>
@@ -25079,7 +25089,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>97.206718329531</v>
@@ -25138,7 +25148,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>96.1759414895127</v>
@@ -25197,7 +25207,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>96.0905023414327</v>
@@ -25256,7 +25266,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>97.4466501672624</v>
@@ -25315,7 +25325,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>96.9078486586345</v>
@@ -25374,7 +25384,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>95.2304353157838</v>
@@ -25433,7 +25443,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>97.7485169969099</v>
@@ -25492,7 +25502,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>96.8620165170747</v>
@@ -25551,7 +25561,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>97.4059974870565</v>
@@ -25610,7 +25620,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>95.9995705222544</v>
@@ -25669,7 +25679,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>95.7932521805545</v>
@@ -25728,7 +25738,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>96.5180185078915</v>
@@ -25787,7 +25797,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>95.7584692737579</v>
@@ -25846,7 +25856,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>98.3942514295879</v>
@@ -25905,7 +25915,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>99.0881669355887</v>
@@ -25964,7 +25974,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>98.2659371888512</v>
@@ -26023,7 +26033,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>99.2337526205684</v>
@@ -26082,7 +26092,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>99.675429351684</v>
@@ -26141,7 +26151,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>97.8083012934341</v>
@@ -26200,7 +26210,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B402" s="2" t="n">
         <v>94.5148820327319</v>
@@ -26259,7 +26269,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B403" s="2" t="n">
         <v>96.0428955043299</v>
@@ -26318,7 +26328,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B404" s="2" t="n">
         <v>97.0825364516256</v>
@@ -26377,7 +26387,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B405" s="2" t="n">
         <v>99.1182102213696</v>
@@ -26436,7 +26446,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B406" s="2" t="n">
         <v>99.3639007697195</v>
@@ -26495,7 +26505,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B407" s="2" t="n">
         <v>98.6137843460634</v>
@@ -26554,7 +26564,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B408" s="2" t="n">
         <v>99.1895156600109</v>
@@ -26613,7 +26623,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B409" s="2" t="n">
         <v>100.069230551496</v>
@@ -26672,7 +26682,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B410" s="2" t="n">
         <v>101.340357290368</v>
@@ -26731,7 +26741,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B411" s="2" t="n">
         <v>101.80337759712</v>
@@ -26790,7 +26800,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B412" s="2" t="n">
         <v>101.592078758007</v>
@@ -26849,7 +26859,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B413" s="2" t="n">
         <v>101.299664818867</v>
@@ -26908,7 +26918,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B414" s="2" t="n">
         <v>103.115184357657</v>
@@ -26967,7 +26977,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B415" s="2" t="n">
         <v>103.158864007317</v>
@@ -27026,7 +27036,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3" t="n">
@@ -27059,7 +27069,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3" t="n">
@@ -27092,7 +27102,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3" t="n">
@@ -27125,7 +27135,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3" t="n">
@@ -27158,7 +27168,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3" t="n">
@@ -27191,7 +27201,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3" t="n">
@@ -27224,7 +27234,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3" t="n">
@@ -27257,7 +27267,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3" t="n">
@@ -27290,7 +27300,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3" t="n">
@@ -27323,7 +27333,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3" t="n">
@@ -27356,7 +27366,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3" t="n">
@@ -27389,7 +27399,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3" t="n">
@@ -27422,7 +27432,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -27445,7 +27455,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -27468,7 +27478,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -27491,7 +27501,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -27514,7 +27524,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -27537,7 +27547,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27560,7 +27570,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27583,7 +27593,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27606,7 +27616,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27629,7 +27639,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27652,7 +27662,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27675,7 +27685,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27698,7 +27708,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27721,7 +27731,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27744,7 +27754,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27767,7 +27777,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27790,7 +27800,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27813,7 +27823,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27836,7 +27846,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27859,7 +27869,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27882,7 +27892,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27905,7 +27915,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27928,7 +27938,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27951,7 +27961,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27974,7 +27984,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -27997,7 +28007,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -28020,7 +28030,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -28043,7 +28053,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -28066,7 +28076,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -28089,7 +28099,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -28112,7 +28122,7 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B458" s="2"/>
       <c r="C458" s="3"/>
@@ -28135,7 +28145,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B459" s="2"/>
       <c r="C459" s="3"/>
@@ -28158,7 +28168,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B460" s="2"/>
       <c r="C460" s="3"/>
@@ -28181,7 +28191,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B461" s="2"/>
       <c r="C461" s="3"/>
@@ -28204,7 +28214,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B462" s="2"/>
       <c r="C462" s="3"/>
@@ -28227,7 +28237,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B463" s="2"/>
       <c r="C463" s="3"/>
@@ -28250,7 +28260,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B464" s="2"/>
       <c r="C464" s="3"/>
@@ -28273,7 +28283,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B465" s="2"/>
       <c r="C465" s="3"/>
@@ -28296,7 +28306,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B466" s="2"/>
       <c r="C466" s="3"/>
@@ -28319,7 +28329,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B467" s="2"/>
       <c r="C467" s="3"/>
@@ -28342,7 +28352,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B468" s="2"/>
       <c r="C468" s="3"/>
@@ -28365,7 +28375,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B469" s="2"/>
       <c r="C469" s="3"/>
@@ -28399,97 +28409,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -28513,7 +28523,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -28523,13 +28533,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.194944619623264</v>
@@ -28537,7 +28547,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.179470879053183</v>
@@ -28545,7 +28555,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.157363303252508</v>
@@ -28553,7 +28563,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.125473994877048</v>
@@ -28561,7 +28571,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.0993542346326295</v>
@@ -28569,7 +28579,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.0922421828552992</v>
@@ -28577,7 +28587,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.100786306683555</v>
@@ -28585,7 +28595,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.117851869682344</v>
@@ -28593,7 +28603,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.148672480844486</v>
@@ -28601,7 +28611,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.178903997210281</v>
@@ -28609,7 +28619,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.196065119802303</v>
@@ -28617,7 +28627,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.178044558539012</v>
@@ -28625,7 +28635,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.120820703307352</v>
@@ -28633,7 +28643,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.0431203427450382</v>
@@ -28641,7 +28651,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0245318166410594</v>
@@ -28649,7 +28659,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.054400501087773</v>
@@ -28657,7 +28667,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.0745016771015152</v>
@@ -28665,7 +28675,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.0969844101243525</v>
@@ -28673,7 +28683,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.0981371576455564</v>

</xml_diff>